<commit_message>
Added new biodiversity corridor, tables, and sampling points
</commit_message>
<xml_diff>
--- a/outputs/sampling_design/block_area_summary.xlsx
+++ b/outputs/sampling_design/block_area_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harre\Repos\CERK\TGBS_Base\outputs\sampling_design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14D694B2-CE90-4C42-9CBD-99DAD46991C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94645703-A321-4DEE-9737-92AD55382A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{583BAF4D-DD18-4518-8402-99E02F54E195}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
   <si>
     <t>Block</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Area_ha</t>
   </si>
   <si>
-    <t>corridor</t>
-  </si>
-  <si>
     <t>Biodiversity Corridor</t>
   </si>
   <si>
@@ -89,6 +86,12 @@
   </si>
   <si>
     <t>23.10557672782341</t>
+  </si>
+  <si>
+    <t>licenced_area_corridor</t>
+  </si>
+  <si>
+    <t>biodiversity_corridor</t>
   </si>
 </sst>
 </file>
@@ -572,9 +575,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -950,9 +956,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{622A47AB-571E-48AC-A728-F9E018E2486A}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="21.36328125" customWidth="1"/>
     <col min="3" max="3" width="21.26953125" customWidth="1"/>
     <col min="4" max="4" width="22.36328125" customWidth="1"/>
   </cols>
@@ -973,209 +980,220 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="2">
+        <v>581.01138749999996</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>1011</v>
-      </c>
-      <c r="B3">
-        <v>2020</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B4">
         <v>2020</v>
       </c>
       <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B5">
         <v>2020</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B6">
         <v>2020</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B7">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B8">
         <v>2021</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>10171</v>
+        <v>1016</v>
       </c>
       <c r="B9">
         <v>2021</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>10181</v>
+        <v>10171</v>
       </c>
       <c r="B10">
         <v>2021</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>10172</v>
+        <v>10181</v>
       </c>
       <c r="B11">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>10182</v>
+        <v>10172</v>
       </c>
       <c r="B12">
         <v>2022</v>
       </c>
       <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>1019</v>
+        <v>10182</v>
       </c>
       <c r="B13">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B14">
         <v>2023</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B15">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B16">
         <v>2024</v>
       </c>
       <c r="C16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1022</v>
+      </c>
+      <c r="B17">
+        <v>2024</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>